<commit_message>
Cierre de la entrega
</commit_message>
<xml_diff>
--- a/docs/tabla_requerimientos_diligenciada.xlsx
+++ b/docs/tabla_requerimientos_diligenciada.xlsx
@@ -85,7 +85,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -105,11 +105,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
@@ -472,7 +467,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -584,22 +579,16 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1264,7 +1253,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="102.4" customHeight="1" s="1" thickBot="1">
+    <row r="9" ht="115.6" customHeight="1" s="1" thickBot="1">
       <c r="A9" s="38" t="n"/>
       <c r="B9" s="6" t="inlineStr">
         <is>
@@ -1288,7 +1277,7 @@
       </c>
       <c r="F9" s="39" t="inlineStr">
         <is>
-          <t>Carga de revisión: en la demo de proporción realista (5,0% de ataque), el Panel de resumen reduce 500 flujos por revisar a 23 alertas priorizadas, es decir, 95,4% menos revisión, y un lote de 50.000 flujos se prioriza en menos de un segundo en local. En lo técnico, el modelo supera con amplitud la línea base trivial que marca todo como normal: macro-F1 de 0,975 frente a 0,082.</t>
+          <t>Carga de revisión: en la demo de proporción realista (5,0% de ataque), el Panel de resumen reduce 500 flujos por revisar a 23 alertas priorizadas, es decir, 95,4% menos revisión, y en local un lote de 50.000 flujos se prioriza en unos 2 s la primera vez y en unos 0,6 s las siguientes. En lo técnico, el modelo supera con amplitud la línea base trivial que marca todo como normal: macro-F1 de 0,975 frente a 0,082.</t>
         </is>
       </c>
       <c r="G9" s="40" t="inlineStr">
@@ -1467,7 +1456,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="89.19999999999999" customHeight="1" s="1">
+    <row r="13" ht="168.4" customHeight="1" s="1">
       <c r="A13" s="34" t="n"/>
       <c r="B13" s="4" t="inlineStr">
         <is>
@@ -1491,33 +1480,33 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Tiempo de respuesta: en local, 50.000 flujos se validan y clasifican en menos de un segundo (entre 0,7 y 0,8 s en mediciones repetidas, con un pico de memoria cercano a 390 MB). La reproducción completa del análisis requiere unos 8 GB de RAM y no usa GPU. [[PENDIENTE: tiempo de 50.000 flujos y volumen máximo estable en el tablero desplegado]]</t>
-        </is>
-      </c>
-      <c r="G13" s="42" t="inlineStr">
-        <is>
-          <t>Pendiente [[PENDIENTE: Cumplido o Cumplido parcialmente según la medición en el desplegado]]</t>
+          <t>Tiempo de respuesta: en el tablero publicado, el lote de 50.000 flujos de tests/generar_lote_r9.py (15,6 MB) se clasificó entre 1,4 y 1,7 s después de terminar la subida (mediana de 1,6 s en tres cargas), frente al límite de 30 s. En local se valida y clasifica en unos 2 s la primera vez en un proceso nuevo (incluye la carga inicial) y en unos 0,6 s las siguientes, con un pico de memoria del proceso de unos 380 MB. No se probaron archivos mayores, para no saturar el alojamiento gratuito compartido, así que el volumen máximo estable por encima de 50.000 flujos no está determinado. La reproducción completa del análisis requiere unos 8 GB de RAM y no usa GPU.</t>
+        </is>
+      </c>
+      <c r="G13" s="36" t="inlineStr">
+        <is>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H13" s="35" t="inlineStr">
         <is>
-          <t>test_R09_local_50000_flujos_en_menos_de_30_segundos (pasa; evidencia parcial, en local).
-Reporte técnico: sección 8.1.
-[[PENDIENTE: medición con archivos de tamaño creciente en el tablero desplegado, empezando por data/interim/lote_r9_50k.csv, que genera tests/generar_lote_r9.py]]</t>
+          <t>Medición en el tablero desplegado el 23 de septiembre de 2026, como visitante anónimo con un perfil limpio de Edge sin interfaz: tres cargas del lote en sesiones nuevas, con 1,68 s, 1,60 s y 1,42 s desde el fin de la subida hasta el aviso de clasificación.
+test_R09_local_50000_flujos_en_menos_de_30_segundos (pasa, en local).
+Reporte técnico: sección 8.1.</t>
         </is>
       </c>
       <c r="I13" s="35" t="inlineStr">
         <is>
-          <t>El tablero carga los modelos una sola vez por servidor y procesa el archivo en memoria. Se preparó un lote de 50.000 flujos para medir en el desplegado.</t>
+          <t>El tablero carga los modelos una sola vez por servidor y procesa el archivo en memoria. Se preparó un lote de 50.000 flujos (tests/generar_lote_r9.py) para medir en el desplegado.</t>
         </is>
       </c>
       <c r="J13" s="37" t="inlineStr">
         <is>
-          <t>Falta la medición en el tablero desplegado, que es la prueba prevista; la medición local es evidencia parcial. Acción correctiva: medir el lote de 50.000 flujos y lotes crecientes en el desplegado. [[PENDIENTE: responsable y fecha]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="62.8" customHeight="1" s="1">
+          <t>No aplica</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="115.6" customHeight="1" s="1">
       <c r="A14" s="34" t="n"/>
       <c r="B14" s="4" t="inlineStr">
         <is>
@@ -1541,28 +1530,29 @@
       </c>
       <c r="F14" s="35" t="inlineStr">
         <is>
-          <t>El tablero está publicado en https://deteccion-trafico-malicioso.streamlit.app/. [[PENDIENTE: acceso a la URL pública desde un equipo distinto al de desarrollo y tiempo de reanudación tras inactividad]]</t>
+          <t>El tablero está publicado en https://deteccion-trafico-malicioso.streamlit.app/, en Streamlit Community Cloud (plan gratuito, Python 3.13), y se abre en el navegador sin instalar nada ni iniciar sesión. Con un perfil de navegador limpio, la URL mostró el tablero listo en unos 7 s y la demo de proporción realista quedó clasificada en menos de 1 s desde el clic.</t>
         </is>
       </c>
       <c r="G14" s="42" t="inlineStr">
         <is>
-          <t>Pendiente [[PENDIENTE: estado según la verificación en el desplegado]]</t>
+          <t>Cumplido parcialmente</t>
         </is>
       </c>
       <c r="H14" s="35" t="inlineStr">
         <is>
-          <t>test_R10_url_publica_responde_y_reanuda_en_menos_de_un_minuto (manual; se omite con su razón).
-[[PENDIENTE: registro de la verificación en el tablero desplegado]]</t>
+          <t>Verificación del 23 de septiembre de 2026 como visitante anónimo, desde el equipo de desarrollo con perfiles limpios de Edge y Chrome sin interfaz: tablero listo en 6,8 s y 6,9 s, y demo realista clasificada en 0,60 s y 0,86 s, sin mensajes de error.
+test_R10_url_publica_responde_y_reanuda_en_menos_de_un_minuto (manual; se omite con su razón).
+Reporte técnico: sección 8.1.</t>
         </is>
       </c>
       <c r="I14" s="35" t="inlineStr">
         <is>
-          <t>requirements.txt liviano, resuelto para Linux, y Python 3.13 fijado para el despliegue.</t>
+          <t>requirements.txt liviano, resuelto para Linux, y Python 3.13 fijado para el despliegue en Streamlit Community Cloud.</t>
         </is>
       </c>
       <c r="J14" s="37" t="inlineStr">
         <is>
-          <t>Depende del despliegue, que aún no existe. Acción correctiva: desplegar el tablero, abrir la URL desde otro equipo y medir la reanudación. [[PENDIENTE: responsable y fecha]]</t>
+          <t>La disponibilidad tiene que sostenerse hasta la calificación en un alojamiento gratuito. Acción correctiva: abrir la URL pública a diario hasta la calificación y confirmar que responde y que reanuda tras un período de inactividad. Responsable: Bryan Rodriguez. Fecha: antes de la presentación ejecutiva.</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1808,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="62.8" customHeight="1" s="1">
+    <row r="20" ht="208" customHeight="1" s="1">
       <c r="A20" s="34" t="n"/>
       <c r="B20" s="4" t="inlineStr">
         <is>
@@ -1842,18 +1832,23 @@
       </c>
       <c r="F20" s="35" t="inlineStr">
         <is>
-          <t>Conteo esperado como criterio: resumen en 1 clic, métricas en 2, explicación de una alerta en 3 y exportación filtrada en 3. [[PENDIENTE: conteo de clics medido en el recorrido del tablero desplegado]]</t>
-        </is>
-      </c>
-      <c r="G20" s="42" t="inlineStr">
-        <is>
-          <t>Pendiente [[PENDIENTE: verificación del recorrido de clics en el tablero desplegado]]</t>
+          <t>Contando desde el tablero recién abierto y sin archivo, el resumen está a 1 clic (Demo de proporción realista), las métricas del modelo a 2 (la demo y Clasificación) y la explicación de la primera alerta de la cola a 2 (Demo rica en ataques e Interpretabilidad). Explicar otra alerta suma 2 clics (abrir el selector y elegirla), y exportar la cola con un filtro toma 4 (la demo, Alertas, un cambio de filtro y la descarga), que son 3 con el archivo ya cargado.</t>
+        </is>
+      </c>
+      <c r="G20" s="36" t="inlineStr">
+        <is>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H20" s="35" t="inlineStr">
         <is>
-          <t>test_R16_resultados_clave_en_tres_clics_o_menos (manual; se omite con su razón, que documenta el conteo esperado).
-[[PENDIENTE: registro del recorrido de clics en el tablero desplegado]]</t>
+          <t>Recorrido en el tablero desplegado el 23 de septiembre de 2026 con clics de ratón (Edge sin interfaz, perfil limpio), cada tarea desde el tablero recién abierto:
+1. Resumen: Demo de proporción realista (1 clic).
+2. Métricas: Demo de proporción realista y Clasificación (2 clics).
+3. Explicación: Demo rica en ataques e Interpretabilidad (2 clics); para otra alerta, además abrir el selector y elegirla (4 clics).
+4. Exportación filtrada: Demo rica en ataques, Alertas, quitar Bot del filtro Tipo de ataque y Descargar estas alertas en CSV (4 clics; el aviso confirmó 174 alertas exportadas).
+test_R16_resultados_clave_en_tres_clics_o_menos (manual; se omite con su razón, que documenta el conteo esperado).
+Reporte técnico: sección 8.1.</t>
         </is>
       </c>
       <c r="I20" s="35" t="inlineStr">
@@ -1863,7 +1858,7 @@
       </c>
       <c r="J20" s="37" t="inlineStr">
         <is>
-          <t>Falta el recorrido contando clics, que es la prueba prevista. Acción correctiva: hacer el recorrido en el tablero desplegado y registrar el conteo. [[PENDIENTE: responsable y fecha]]</t>
+          <t>No aplica</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2012,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="52.05" customHeight="1" s="1">
+    <row r="24" ht="62.8" customHeight="1" s="1">
       <c r="A24" s="7" t="inlineStr">
         <is>
           <t>USABILIDAD</t>
@@ -2045,18 +2040,18 @@
       </c>
       <c r="F24" s="31" t="inlineStr">
         <is>
-          <t>[[PENDIENTE: resultado de la prueba con una persona ajena al proyecto y sin conocimientos de programación (cargar archivo, revisar alertas y exportar)]]</t>
-        </is>
-      </c>
-      <c r="G24" s="45" t="inlineStr">
-        <is>
-          <t>Pendiente [[PENDIENTE: estado según la prueba de usabilidad]]</t>
+          <t>Operación sin conocimientos técnicos: una persona ajena al proyecto y sin formación técnica completó sin asistencia, en el tablero desplegado, el recorrido de cargar una demo, revisar las alertas y exportarlas.</t>
+        </is>
+      </c>
+      <c r="G24" s="32" t="inlineStr">
+        <is>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H24" s="31" t="inlineStr">
         <is>
-          <t>test_R20_usuario_ajeno_completa_el_recorrido_sin_ayuda (manual; se omite con su razón).
-[[PENDIENTE: registro de la prueba de usabilidad]]</t>
+          <t>Prueba realizada el 23 de septiembre de 2026 en el tablero desplegado, informada por Bryan Rodriguez.
+test_R20_usuario_ajeno_completa_el_recorrido_sin_ayuda (manual; se omite con su razón).</t>
         </is>
       </c>
       <c r="I24" s="31" t="inlineStr">
@@ -2066,11 +2061,11 @@
       </c>
       <c r="J24" s="33" t="inlineStr">
         <is>
-          <t>Requiere una persona ajena al proyecto y se hará sobre el tablero desplegado. [[PENDIENTE: responsable y fecha]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="102.4" customHeight="1" s="1">
+          <t>No aplica</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="115.6" customHeight="1" s="1">
       <c r="A25" s="34" t="n"/>
       <c r="B25" s="4" t="inlineStr">
         <is>
@@ -2094,19 +2089,20 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Las seis pantallas abren con su título y una descripción de lo que muestran, las pantallas con tablas traen su guía "Cómo leer" y los términos técnicos de las métricas (macro-F1, recall, precisión, SHAP y score de anomalía) se explican en lenguaje llano en la misma pantalla donde aparecen. [[PENDIENTE: resultado de la revisión de los textos por una persona ajena al proyecto]]</t>
-        </is>
-      </c>
-      <c r="G25" s="46" t="inlineStr">
-        <is>
-          <t>Cumplido parcialmente [[PENDIENTE: estado final tras la revisión por una persona ajena]]</t>
+          <t>Las seis pantallas abren con su título y una descripción de lo que muestran, las pantallas con tablas traen su guía "Cómo leer" y los términos técnicos de las métricas (macro-F1, recall, precisión, SHAP y score de anomalía) se explican en lenguaje llano en la misma pantalla donde aparecen. El tablero se mostró a 3 personas y todas pudieron comprender su funcionamiento.</t>
+        </is>
+      </c>
+      <c r="G25" s="42" t="inlineStr">
+        <is>
+          <t>Cumplido parcialmente</t>
         </is>
       </c>
       <c r="H25" s="35" t="inlineStr">
         <is>
           <t>test_R21_cada_pantalla_dice_que_muestra_y_como_leerlo (pasa): revisa el código de las seis pantallas.
-test_R21_revision_de_textos_por_persona_ajena (manual; se omite con su razón).
-[[PENDIENTE: registro de la revisión de textos]]</t>
+Prueba de usabilidad del 23 de septiembre de 2026 (ver R20): una persona ajena completó el recorrido sin asistencia.
+Se mostró el tablero a 3 personas y todas pudieron comprender su funcionamiento.
+test_R21_revision_de_textos_por_persona_ajena (manual; se omite con su razón).</t>
         </is>
       </c>
       <c r="I25" s="35" t="inlineStr">
@@ -2116,11 +2112,11 @@
       </c>
       <c r="J25" s="37" t="inlineStr">
         <is>
-          <t>Falta la revisión por una persona ajena al proyecto, que es la prueba prevista. [[PENDIENTE: responsable y fecha]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="62.8" customHeight="1" s="1" thickBot="1">
+          <t>Falta la revisión formal de los textos por una persona ajena al proyecto, que es la prueba prevista. Acción correctiva: hacer esa revisión pantalla por pantalla y corregir lo que no se entienda. Responsable: Bryan Rodriguez. Fecha: antes de la presentación ejecutiva.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="115.6" customHeight="1" s="1" thickBot="1">
       <c r="A26" s="38" t="n"/>
       <c r="B26" s="6" t="inlineStr">
         <is>
@@ -2142,30 +2138,31 @@
           <t>Funciona en navegadores de escritorio modernos; el usuario solo necesita la URL. No optimizado para dispositivos móviles.</t>
         </is>
       </c>
-      <c r="F26" s="47" t="inlineStr">
-        <is>
-          <t>[[PENDIENTE: apertura del tablero desplegado en Chrome, Firefox y Edge de escritorio]]</t>
-        </is>
-      </c>
-      <c r="G26" s="48" t="inlineStr">
-        <is>
-          <t>Pendiente [[PENDIENTE: estado según la verificación en los tres navegadores]]</t>
-        </is>
-      </c>
-      <c r="H26" s="47" t="inlineStr">
-        <is>
-          <t>test_R22_funciona_en_chrome_firefox_y_edge (manual; se omite con su razón).
-[[PENDIENTE: registro de la verificación en el tablero desplegado]]</t>
-        </is>
-      </c>
-      <c r="I26" s="47" t="inlineStr">
+      <c r="F26" s="45" t="inlineStr">
+        <is>
+          <t>Compatibilidad de acceso: el tablero desplegado se abrió con solo la URL, sin instalación ni configuración, y sus seis pantallas cargaron con la demo rica, con su título y sin mensajes de error, en Edge 153, Chrome 153 y el motor de Firefox 155. No está optimizado para dispositivos móviles, como se declara en el manual.</t>
+        </is>
+      </c>
+      <c r="G26" s="46" t="inlineStr">
+        <is>
+          <t>Cumplido</t>
+        </is>
+      </c>
+      <c r="H26" s="45" t="inlineStr">
+        <is>
+          <t>Verificación del 23 de septiembre de 2026 como visitante anónimo, con perfiles limpios: Edge 153 y Chrome 153 instalados en el equipo, ejecutados sin interfaz, y el motor de Firefox 155 que distribuye la biblioteca de automatización Playwright (no la aplicación de escritorio de Firefox).
+test_R22_funciona_en_chrome_firefox_y_edge (manual; se omite con su razón).
+Reporte técnico: sección 8.1.</t>
+        </is>
+      </c>
+      <c r="I26" s="45" t="inlineStr">
         <is>
           <t>El tablero solo necesita la URL; no requiere instalación ni configuración del navegador. Se declara que no está optimizado para dispositivos móviles.</t>
         </is>
       </c>
-      <c r="J26" s="49" t="inlineStr">
-        <is>
-          <t>Depende del despliegue. Acción correctiva: abrir el tablero desplegado en los tres navegadores y registrar el resultado. [[PENDIENTE: responsable y fecha]]</t>
+      <c r="J26" s="47" t="inlineStr">
+        <is>
+          <t>No aplica</t>
         </is>
       </c>
     </row>
@@ -2187,9 +2184,9 @@
           <t>Por qué queda fuera</t>
         </is>
       </c>
-      <c r="C29" s="50" t="n"/>
-      <c r="D29" s="50" t="n"/>
-      <c r="E29" s="51" t="n"/>
+      <c r="C29" s="48" t="n"/>
+      <c r="D29" s="48" t="n"/>
+      <c r="E29" s="49" t="n"/>
     </row>
     <row r="30" ht="30" customHeight="1" s="1">
       <c r="A30" s="20" t="inlineStr">
@@ -2202,9 +2199,9 @@
           <t>Requiere librerías y tiempo adicionales, la exportación en CSV cubre la necesidad.</t>
         </is>
       </c>
-      <c r="C30" s="50" t="n"/>
-      <c r="D30" s="50" t="n"/>
-      <c r="E30" s="51" t="n"/>
+      <c r="C30" s="48" t="n"/>
+      <c r="D30" s="48" t="n"/>
+      <c r="E30" s="49" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1" s="1">
       <c r="A31" s="20" t="inlineStr">
@@ -2217,9 +2214,9 @@
           <t>El hosting gratuito no garantiza la persistencia de archivos entre reinicios.</t>
         </is>
       </c>
-      <c r="C31" s="50" t="n"/>
-      <c r="D31" s="50" t="n"/>
-      <c r="E31" s="51" t="n"/>
+      <c r="C31" s="48" t="n"/>
+      <c r="D31" s="48" t="n"/>
+      <c r="E31" s="49" t="n"/>
     </row>
     <row r="32" ht="30" customHeight="1" s="1">
       <c r="A32" s="20" t="inlineStr">
@@ -2232,9 +2229,9 @@
           <t>Requiere características agregadas por ventana de tiempo: el flujo individual no contiene la señal.</t>
         </is>
       </c>
-      <c r="C32" s="50" t="n"/>
-      <c r="D32" s="50" t="n"/>
-      <c r="E32" s="51" t="n"/>
+      <c r="C32" s="48" t="n"/>
+      <c r="D32" s="48" t="n"/>
+      <c r="E32" s="49" t="n"/>
     </row>
     <row r="33" ht="30" customHeight="1" s="1">
       <c r="A33" s="20" t="inlineStr">
@@ -2247,9 +2244,9 @@
           <t>652 y 21 casos respectivamente: insuficientes para métricas por clase confiables.</t>
         </is>
       </c>
-      <c r="C33" s="50" t="n"/>
-      <c r="D33" s="50" t="n"/>
-      <c r="E33" s="51" t="n"/>
+      <c r="C33" s="48" t="n"/>
+      <c r="D33" s="48" t="n"/>
+      <c r="E33" s="49" t="n"/>
     </row>
     <row r="34" ht="30" customHeight="1" s="1">
       <c r="A34" s="20" t="inlineStr">
@@ -2262,9 +2259,9 @@
           <t>Resolvería la fragilidad del umbral de operación observada en la evaluación final.</t>
         </is>
       </c>
-      <c r="C34" s="50" t="n"/>
-      <c r="D34" s="50" t="n"/>
-      <c r="E34" s="51" t="n"/>
+      <c r="C34" s="48" t="n"/>
+      <c r="D34" s="48" t="n"/>
+      <c r="E34" s="49" t="n"/>
     </row>
     <row r="35" ht="30" customHeight="1" s="1">
       <c r="A35" s="20" t="inlineStr">
@@ -2277,9 +2274,9 @@
           <t>El prototipo opera por lotes sobre archivos cargados por el usuario.</t>
         </is>
       </c>
-      <c r="C35" s="50" t="n"/>
-      <c r="D35" s="50" t="n"/>
-      <c r="E35" s="51" t="n"/>
+      <c r="C35" s="48" t="n"/>
+      <c r="D35" s="48" t="n"/>
+      <c r="E35" s="49" t="n"/>
     </row>
     <row r="36" ht="30" customHeight="1" s="1">
       <c r="A36" s="20" t="inlineStr">
@@ -2292,9 +2289,9 @@
           <t>Requiere una escala de severidad definida y justificada por criterio de dominio.</t>
         </is>
       </c>
-      <c r="C36" s="50" t="n"/>
-      <c r="D36" s="50" t="n"/>
-      <c r="E36" s="51" t="n"/>
+      <c r="C36" s="48" t="n"/>
+      <c r="D36" s="48" t="n"/>
+      <c r="E36" s="49" t="n"/>
     </row>
     <row r="38" ht="40" customHeight="1" s="1">
       <c r="A38" s="2" t="inlineStr">

</xml_diff>